<commit_message>
Fix CSV encoding fallback; tidy tests
</commit_message>
<xml_diff>
--- a/reports/comparison_report.xlsx
+++ b/reports/comparison_report.xlsx
@@ -436,7 +436,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Rows (src / tgt)  : 3 / 4</t>
+          <t>Rows (src / tgt)  : 254045 / 254044</t>
         </is>
       </c>
     </row>
@@ -464,14 +464,14 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Only in source    : 0 rows</t>
+          <t>Only in source    : 1 rows</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Only in target    : 1 rows</t>
+          <t>Only in target    : 0 rows</t>
         </is>
       </c>
     </row>
@@ -493,7 +493,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -504,12 +504,79 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>NAME</t>
+          <t>FIRST_NAME</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>LAST_NAME</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>EMAIL</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>AGE</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
           <t>CITY</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>SALARY</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>JOINED</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>254045</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Jane</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Johnson</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>jane.johnson254045@mail.co</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Dover</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>129369.17</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>2016-06-08</t>
         </is>
       </c>
     </row>
@@ -524,7 +591,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -535,29 +602,37 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>NAME</t>
+          <t>FIRST_NAME</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>LAST_NAME</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>EMAIL</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>AGE</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
           <t>CITY</t>
         </is>
       </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Kiran</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Goa</t>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>SALARY</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>JOINED</t>
         </is>
       </c>
     </row>
@@ -600,7 +675,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -610,12 +685,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Delhi</t>
+          <t>Riverside</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Mumbai</t>
+          <t>CHANGED_BY_TEST</t>
         </is>
       </c>
     </row>

</xml_diff>